<commit_message>
Fix NDT billing records save error (config_manager module not found) and update work history
</commit_message>
<xml_diff>
--- a/home/src/site_apps/central/data/Material_Inventory.xlsx
+++ b/home/src/site_apps/central/data/Material_Inventory.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Materials" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Budget" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Settings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26066,7 +26066,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -26077,11 +26077,11 @@
         <v>480</v>
       </c>
       <c r="D5" t="n">
-        <v>4.4686</v>
+        <v>17.8744</v>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" s="1" t="n">
-        <v>46272.70826592592</v>
+        <v>46272.70844920139</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -26115,7 +26115,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>4.4686</v>
+        <v>17.8744</v>
       </c>
       <c r="Q5" t="n">
         <v>201863</v>
@@ -26127,7 +26127,7 @@
         <v>0</v>
       </c>
       <c r="T5" t="n">
-        <v>902045</v>
+        <v>3608180</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
@@ -26139,21 +26139,29 @@
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>(주간) 09:00~18:00</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr"/>
+          <t>(휴일) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>67,500</t>
+        </is>
+      </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>부장 박광복</t>
+          <t>계장 이준우</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>(주간) 09:00~18:00</t>
-        </is>
-      </c>
-      <c r="AA5" t="inlineStr"/>
+          <t>(휴일) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>67,500</t>
+        </is>
+      </c>
       <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="inlineStr"/>
       <c r="AD5" t="inlineStr"/>
@@ -26263,19 +26271,19 @@
         <v>1</v>
       </c>
       <c r="CH5" t="n">
-        <v>4.4686</v>
+        <v>17.8744</v>
       </c>
       <c r="CI5" t="n">
-        <v>167836</v>
+        <v>671344</v>
       </c>
       <c r="CJ5" t="n">
-        <v>291352</v>
+        <v>1165410</v>
       </c>
       <c r="CK5" t="n">
-        <v>320487</v>
+        <v>1281951</v>
       </c>
       <c r="CL5" t="n">
-        <v>122368</v>
+        <v>489472</v>
       </c>
       <c r="CM5" t="inlineStr"/>
       <c r="CN5" t="inlineStr"/>
@@ -26293,7 +26301,7 @@
         </is>
       </c>
       <c r="CX5" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="CY5" t="n">
         <v>0</v>
@@ -26317,7 +26325,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46270</v>
+        <v>46268</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -26328,11 +26336,11 @@
         <v>480</v>
       </c>
       <c r="D6" t="n">
-        <v>17.8744</v>
+        <v>4.4686</v>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" s="1" t="n">
-        <v>46272.70844920139</v>
+        <v>46273.01988914352</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -26366,7 +26374,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>17.8744</v>
+        <v>4.4686</v>
       </c>
       <c r="Q6" t="n">
         <v>201863</v>
@@ -26378,7 +26386,7 @@
         <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>3608180</v>
+        <v>902045</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
@@ -26390,29 +26398,21 @@
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>(휴일) 09:00~18:00</t>
-        </is>
-      </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>67,500</t>
-        </is>
-      </c>
+          <t>(주간) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr"/>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>계장 이준우</t>
+          <t>부장 박광복</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>(휴일) 09:00~18:00</t>
-        </is>
-      </c>
-      <c r="AA6" t="inlineStr">
-        <is>
-          <t>67,500</t>
-        </is>
-      </c>
+          <t>(주간) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr"/>
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr"/>
       <c r="AD6" t="inlineStr"/>
@@ -26522,19 +26522,19 @@
         <v>1</v>
       </c>
       <c r="CH6" t="n">
-        <v>17.8744</v>
+        <v>0</v>
       </c>
       <c r="CI6" t="n">
-        <v>671344</v>
+        <v>0</v>
       </c>
       <c r="CJ6" t="n">
-        <v>1165410</v>
+        <v>0</v>
       </c>
       <c r="CK6" t="n">
-        <v>1281951</v>
+        <v>0</v>
       </c>
       <c r="CL6" t="n">
-        <v>489472</v>
+        <v>0</v>
       </c>
       <c r="CM6" t="inlineStr"/>
       <c r="CN6" t="inlineStr"/>
@@ -26552,7 +26552,7 @@
         </is>
       </c>
       <c r="CX6" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="CY6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
fix(billing): correct Excel export sum logic and formatting
</commit_message>
<xml_diff>
--- a/home/src/site_apps/central/data/Material_Inventory.xlsx
+++ b/home/src/site_apps/central/data/Material_Inventory.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Materials" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Budget" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Settings" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24725,7 +24725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DE6"/>
+  <dimension ref="A1:DE8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26574,6 +26574,556 @@
         <v>0</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>중앙지사</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>480</v>
+      </c>
+      <c r="D7" t="n">
+        <v>17.8744</v>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" s="1" t="n">
+        <v>46277.52000121528</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>PAUT MX2(OMNI2-103085)</t>
+        </is>
+      </c>
+      <c r="P7" t="n">
+        <v>17.8744</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>201863</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" t="n">
+        <v>3608180</v>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>PAUT</t>
+        </is>
+      </c>
+      <c r="V7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~22:00</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>16,000</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>부장 박광복</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~22:00</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>16,000</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>계장 이준우</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~22:00</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>16,000</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr"/>
+      <c r="AK7" t="inlineStr"/>
+      <c r="AL7" t="inlineStr"/>
+      <c r="AM7" t="inlineStr"/>
+      <c r="AN7" t="inlineStr"/>
+      <c r="AO7" t="inlineStr"/>
+      <c r="AP7" t="inlineStr"/>
+      <c r="AQ7" t="inlineStr"/>
+      <c r="AR7" t="inlineStr"/>
+      <c r="AS7" t="inlineStr"/>
+      <c r="AT7" t="inlineStr"/>
+      <c r="AU7" t="inlineStr"/>
+      <c r="AV7" t="inlineStr"/>
+      <c r="AW7" t="inlineStr"/>
+      <c r="AX7" t="inlineStr"/>
+      <c r="AY7" t="inlineStr"/>
+      <c r="AZ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG7" t="inlineStr">
+        <is>
+          <t>95가0175 (스타렉스)</t>
+        </is>
+      </c>
+      <c r="BH7" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="BI7" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
+        </is>
+      </c>
+      <c r="BJ7" t="inlineStr"/>
+      <c r="BK7" t="inlineStr"/>
+      <c r="BL7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM7" t="inlineStr"/>
+      <c r="BN7" t="inlineStr">
+        <is>
+          <t>한국지역난방공사 중앙지사</t>
+        </is>
+      </c>
+      <c r="BO7" t="inlineStr"/>
+      <c r="BP7" t="inlineStr"/>
+      <c r="BQ7" t="inlineStr"/>
+      <c r="BR7" t="inlineStr"/>
+      <c r="BS7" t="inlineStr"/>
+      <c r="BT7" t="inlineStr"/>
+      <c r="BU7" t="inlineStr"/>
+      <c r="BV7" t="inlineStr">
+        <is>
+          <t>Pipe</t>
+        </is>
+      </c>
+      <c r="BW7" t="inlineStr">
+        <is>
+          <t>KS B ISO 13588</t>
+        </is>
+      </c>
+      <c r="BX7" t="inlineStr"/>
+      <c r="BY7" t="inlineStr"/>
+      <c r="BZ7" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="CA7" t="inlineStr"/>
+      <c r="CB7" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC7" t="inlineStr">
+        <is>
+          <t>300A 이상 (1.0)</t>
+        </is>
+      </c>
+      <c r="CD7" t="inlineStr"/>
+      <c r="CE7" t="inlineStr"/>
+      <c r="CF7" t="inlineStr"/>
+      <c r="CG7" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH7" t="n">
+        <v>17.8744</v>
+      </c>
+      <c r="CI7" t="n">
+        <v>671344</v>
+      </c>
+      <c r="CJ7" t="n">
+        <v>1165410</v>
+      </c>
+      <c r="CK7" t="n">
+        <v>1281951</v>
+      </c>
+      <c r="CL7" t="n">
+        <v>489472</v>
+      </c>
+      <c r="CM7" t="inlineStr"/>
+      <c r="CN7" t="inlineStr"/>
+      <c r="CO7" t="inlineStr"/>
+      <c r="CP7" t="inlineStr"/>
+      <c r="CQ7" t="inlineStr"/>
+      <c r="CR7" t="inlineStr"/>
+      <c r="CS7" t="inlineStr"/>
+      <c r="CT7" t="inlineStr"/>
+      <c r="CU7" t="inlineStr"/>
+      <c r="CV7" t="inlineStr"/>
+      <c r="CW7" t="inlineStr">
+        <is>
+          <t>ORI</t>
+        </is>
+      </c>
+      <c r="CX7" t="n">
+        <v>8</v>
+      </c>
+      <c r="CY7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ7" t="inlineStr">
+        <is>
+          <t>700A</t>
+        </is>
+      </c>
+      <c r="DA7" t="inlineStr">
+        <is>
+          <t>열배관</t>
+        </is>
+      </c>
+      <c r="DB7" t="inlineStr"/>
+      <c r="DC7" t="inlineStr"/>
+      <c r="DD7" t="inlineStr"/>
+      <c r="DE7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>46273</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>중앙지사</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>480</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2.0385</v>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" s="1" t="n">
+        <v>46277.52028597222</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>PAUT MX2(OMNI2-103085)</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
+        <v>2.0385</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>201863</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" t="n">
+        <v>411497</v>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>PAUT</t>
+        </is>
+      </c>
+      <c r="V8" t="n">
+        <v>0</v>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~22:00</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>16,000</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>부장 박광복</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~22:00</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>16,000</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>계장 이준우</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~22:00</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>16,000</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr"/>
+      <c r="AG8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
+      <c r="AJ8" t="inlineStr"/>
+      <c r="AK8" t="inlineStr"/>
+      <c r="AL8" t="inlineStr"/>
+      <c r="AM8" t="inlineStr"/>
+      <c r="AN8" t="inlineStr"/>
+      <c r="AO8" t="inlineStr"/>
+      <c r="AP8" t="inlineStr"/>
+      <c r="AQ8" t="inlineStr"/>
+      <c r="AR8" t="inlineStr"/>
+      <c r="AS8" t="inlineStr"/>
+      <c r="AT8" t="inlineStr"/>
+      <c r="AU8" t="inlineStr"/>
+      <c r="AV8" t="inlineStr"/>
+      <c r="AW8" t="inlineStr"/>
+      <c r="AX8" t="inlineStr"/>
+      <c r="AY8" t="inlineStr"/>
+      <c r="AZ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG8" t="inlineStr">
+        <is>
+          <t>95가0175 (스타렉스)</t>
+        </is>
+      </c>
+      <c r="BH8" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="BI8" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
+        </is>
+      </c>
+      <c r="BJ8" t="inlineStr"/>
+      <c r="BK8" t="inlineStr"/>
+      <c r="BL8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM8" t="inlineStr"/>
+      <c r="BN8" t="inlineStr">
+        <is>
+          <t>한국지역난방공사 중앙지사</t>
+        </is>
+      </c>
+      <c r="BO8" t="inlineStr"/>
+      <c r="BP8" t="inlineStr"/>
+      <c r="BQ8" t="inlineStr"/>
+      <c r="BR8" t="inlineStr"/>
+      <c r="BS8" t="inlineStr"/>
+      <c r="BT8" t="inlineStr"/>
+      <c r="BU8" t="inlineStr"/>
+      <c r="BV8" t="inlineStr">
+        <is>
+          <t>Pipe</t>
+        </is>
+      </c>
+      <c r="BW8" t="inlineStr">
+        <is>
+          <t>KS B ISO 13588</t>
+        </is>
+      </c>
+      <c r="BX8" t="inlineStr"/>
+      <c r="BY8" t="inlineStr"/>
+      <c r="BZ8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="CA8" t="inlineStr"/>
+      <c r="CB8" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC8" t="inlineStr">
+        <is>
+          <t>300A 이상 (1.0)</t>
+        </is>
+      </c>
+      <c r="CD8" t="inlineStr"/>
+      <c r="CE8" t="inlineStr"/>
+      <c r="CF8" t="inlineStr"/>
+      <c r="CG8" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH8" t="n">
+        <v>2.0385</v>
+      </c>
+      <c r="CI8" t="n">
+        <v>76564</v>
+      </c>
+      <c r="CJ8" t="n">
+        <v>132910</v>
+      </c>
+      <c r="CK8" t="n">
+        <v>146201</v>
+      </c>
+      <c r="CL8" t="n">
+        <v>55822</v>
+      </c>
+      <c r="CM8" t="inlineStr"/>
+      <c r="CN8" t="inlineStr"/>
+      <c r="CO8" t="inlineStr"/>
+      <c r="CP8" t="inlineStr"/>
+      <c r="CQ8" t="inlineStr"/>
+      <c r="CR8" t="inlineStr"/>
+      <c r="CS8" t="inlineStr"/>
+      <c r="CT8" t="inlineStr"/>
+      <c r="CU8" t="inlineStr"/>
+      <c r="CV8" t="inlineStr"/>
+      <c r="CW8" t="inlineStr">
+        <is>
+          <t>ORI</t>
+        </is>
+      </c>
+      <c r="CX8" t="n">
+        <v>3</v>
+      </c>
+      <c r="CY8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ8" t="inlineStr">
+        <is>
+          <t>200A</t>
+        </is>
+      </c>
+      <c r="DA8" t="inlineStr">
+        <is>
+          <t>열배관</t>
+        </is>
+      </c>
+      <c r="DB8" t="inlineStr"/>
+      <c r="DC8" t="inlineStr"/>
+      <c r="DD8" t="inlineStr"/>
+      <c r="DE8" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -26585,7 +27135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y2"/>
+  <dimension ref="A1:Y3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26799,6 +27349,93 @@
       <c r="Y2" t="inlineStr">
         <is>
           <t>{"site_expense": [{"cat": "\ucc28\ub7c9\uc720\uc9c0\ube44", "cont": "\uc8fc\uc720, \uc218\ub9ac, \ud1b5\ud589, \uc8fc\ucc28 \ub4f1", "ppl": "N/A", "qty": "6", "unit": "\uc77c", "price": "6667", "amount": "40,002"}, {"cat": "\uc18c\ubaa8\ud488\ube44", "cont": "\uc7a5\uac11,\uc77c\ud68c\uc6a9 \uc791\uc5c5\ubcf5\uc678", "ppl": "N/A", "qty": "6", "unit": "\uc77c", "price": "3333", "amount": "19,998"}, {"cat": "\ubcf5\ub9ac\ud6c4\uc0dd\ube44", "cont": "\uc0dd\uc218, \uc74c\ub8cc \uc678 \uae30\ud0c0", "ppl": "N/A", "qty": "6", "unit": "\uc77c", "price": "1667", "amount": "10,002"}, {"cat": "Se-175", "cont": "\ubc29\uc0ac\uc131\ub3d9\uc704\uc6d0\uc18c \uad6c\ub9e4", "ppl": "N/A", "qty": "", "unit": "\uc77c", "price": "35,714", "amount": "0"}], "rental": [{"cat": "", "spec": "", "qty": "", "period": "", "unit": "", "price": "0", "amount": "0"}, {"cat": "", "spec": "", "qty": "", "period": "", "unit": "", "price": "0", "amount": "0"}, {"cat": "", "spec": "", "qty": "", "period": "", "unit": "", "price": "0", "amount": "0"}], "outsource": [{"cat": "\ucf00\uc774\uc5d4\ub514\uc774", "work": "\ubc29\uc0ac\uc120\ud22c\uacfc\uac80\uc0ac", "count": "0", "price": "0", "amount": "0"}, {"cat": "", "work": "", "count": "0", "price": "0", "amount": "0"}, {"cat": "", "work": "", "count": "0", "price": "0", "amount": "0"}], "depreciation": [{"item": "PAUT \uc7a5\ube44", "spec": "", "life": "5", "qty": "1", "days": "5", "rate": "44,444", "amount": "222,222"}, {"item": "PAUT SCANNER (MANUAL)", "spec": "", "life": "5", "qty": "1", "days": "5", "rate": "5,556", "amount": "27,778"}, {"item": "PAUT SCANNER (COBRA)", "spec": "", "life": "5", "qty": "1", "days": "", "rate": "16,667", "amount": "0"}, {"item": "YOKE", "spec": "", "life": "5", "qty": "1", "days": "", "rate": "222", "amount": "0"}, {"item": "\ud604\uc0c1\uc6a9 \ud0d1\ucc28(5\ub144\uac04 \ubcf4\ud5d8\ube44 \ud3ec\ud568)", "spec": "\ud604\uc7a5\ubcc4 \ucc28\ub7c9\uae30\uc785\uc2dc \ud0d1\ucc28 \uad6c\ubd84 \uae30\uc785", "life": "5", "qty": "1", "days": "", "rate": "16,667", "amount": "0"}, {"item": "\uc2a4\ud0c0\ub809\uc2a4(5\ub144\uac04 \ubcf4\ud5d8\ube44 \ud3ec\ud568)", "spec": "\ud604\uc7a5\ubcc4 \ucc28\ub7c9\uae30\uc785\uc2dc \uc2a4\ud0c0\ub809\uc2a4 \uad6c\ubd84 \uae30\uc785", "life": "5", "qty": "1", "days": "6", "rate": "16,667", "amount": "100,000"}], "_depreciation_precise_rates": [44444.441666666666, 5555.558333333333, 16666.666666666668, 222.2, 16666.666666666668, 16666.66875]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>0</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>{"\uc774\uc0ac": {"personnel": "", "period": "", "unit_price": 230208.33333333334}, "\ubd80\uc7a5": {"personnel": "1", "period": "160", "unit_price": 230208.33333333334}, "\ucc28\uc7a5": {"personnel": "1", "period": "120", "unit_price": 198625.0}, "\uacfc\uc7a5": {"personnel": "", "period": "", "unit_price": 171541.66666666666}, "\ub300\ub9ac": {"personnel": "1", "period": "160", "unit_price": 158000.0}, "\uacc4\uc7a5": {"personnel": "1", "period": "120", "unit_price": 144458.33333333334}, "\uc8fc\uc784": {"personnel": "", "period": "", "unit_price": 130916.66666666667}, "\uae30\uc0ac": {"personnel": "", "period": "", "unit_price": 121875.0}, "\uc5f0\uc7a5\uadfc\ubb34": {"personnel": "4", "period": "60", "unit_price": 4000.0}, "\uc57c\uac04\uadfc\ubb34": {"personnel": "4", "period": "60", "unit_price": 5000.0}, "\ud734\uc77c\uadfc\ubb34": {"personnel": "4", "period": "62", "unit_price": 7500.0}}</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>[{"qty": "10", "price": "2,200"}, {"qty": "1", "price": "2,950"}, {"qty": "10", "price": "2,700"}, {"qty": "10", "price": "3,000"}, {"qty": "10", "price": "2,600"}, {"qty": "490", "price": "1,700"}, {"qty": "2", "price": "100,000"}, {"qty": "6", "price": "23,000"}, {"qty": "6", "price": "23,000"}, {"qty": "6", "price": "3,500"}, {"qty": "1", "price": "10300000"}]</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>{"site_expense": [{"cat": "\ucc28\ub7c9\uc720\uc9c0\ube44", "cont": "\uc8fc\uc720, \uc218\ub9ac, \ud1b5\ud589, \uc8fc\ucc28 \ub4f1", "ppl": "N/A", "qty": "12", "unit": "\uac1c\uc6d4", "price": "200,000", "amount": "2,400,000"}, {"cat": "\uc18c\ubaa8\ud488\ube44", "cont": "\uc7a5\uac11,\uc77c\ud68c\uc6a9 \uc791\uc5c5\ubcf5\uc678", "ppl": "N/A", "qty": "12", "unit": "\uac1c\uc6d4", "price": "100,000", "amount": "1,200,000"}, {"cat": "\ubcf5\ub9ac\ud6c4\uc0dd\ube44", "cont": "\uc0dd\uc218, \uc74c\ub8cc \uc678 \uae30\ud0c0", "ppl": "N/A", "qty": "12", "unit": "\uac1c\uc6d4", "price": "50,000", "amount": "600,000"}], "rental": [{"cat": "", "spec": "", "qty": "", "period": "", "unit": "", "price": "0", "amount": "0"}, {"cat": "", "spec": "", "qty": "", "period": "", "unit": "", "price": "0", "amount": "0"}, {"cat": "", "spec": "", "qty": "", "period": "", "unit": "", "price": "0", "amount": "0"}], "outsource": [{"cat": "\ucf00\uc774\uc5d4\ub514\uc544\uc774", "work": "\ubc29\uc0ac\uc120\ud22c\uacfc\uac80\uc0ac", "count": "0", "price": "0", "amount": "0"}, {"cat": "", "work": "", "count": "0", "price": "0", "amount": "0"}, {"cat": "", "work": "", "count": "0", "price": "0", "amount": "0"}], "depreciation": [{"item": "PAUT \uc7a5\ube44", "spec": "", "life": "5", "qty": "1", "days": "120", "rate": "44,444", "amount": "5,333,333"}, {"item": "PAUT SCANNER (MANUAL)", "spec": "", "life": "5", "qty": "1", "days": "120", "rate": "5,556", "amount": "666,667"}, {"item": "PAUT SCANNER (COBRA)", "spec": "", "life": "5", "qty": "1", "days": "120", "rate": "16,667", "amount": "2,000,000"}, {"item": "YOKE", "spec": "", "life": "5", "qty": "1", "days": "10", "rate": "222", "amount": "2,222"}, {"item": "\ud604\uc7a5\uc6a9 \ud0d1\ucc28(5\ub144\uac04 \ubcf4\ud5d8\ube44 \ud3ec\ud568)", "spec": "", "life": "5", "qty": "1", "days": "30", "rate": "16,667", "amount": "500,000"}, {"item": "\uc2a4\ud0c0\ub809\uc2a4(5\ub144\uac04 \ubcf4\ud5d8\ube44 \ud3ec\ud568)", "spec": "", "life": "5", "qty": "1", "days": "160", "rate": "16,667", "amount": "2,666,667"}], "_depreciation_precise_rates": [44444.441666666666, 5555.558333333333, 16666.666666666668, 222.2, 16666.666666666668, 16666.66875]}</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>전체</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>288268000</v>
+      </c>
+      <c r="G3" t="n">
+        <v>107303333</v>
+      </c>
+      <c r="H3" t="n">
+        <v>11737950</v>
+      </c>
+      <c r="I3" t="n">
+        <v>27144786</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>142081931</v>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="n">
+        <v>13461323</v>
+      </c>
+      <c r="N3" t="n">
+        <v>13461323</v>
+      </c>
+      <c r="O3" t="n">
+        <v>3268210</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>1722002</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>2026.08.04~2027.08.05</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>{"\uc774\uc0ac": {"personnel": "", "period": "", "unit_price": 230208.33333333334}, "\ubd80\uc7a5": {"personnel": "2", "period": "5.5", "unit_price": 230208.33333333334}, "\ucc28\uc7a5": {"personnel": "", "period": "", "unit_price": 198625.0}, "\uacfc\uc7a5": {"personnel": "", "period": "", "unit_price": 171541.66666666666}, "\ub300\ub9ac": {"personnel": "", "period": "", "unit_price": 158000.0}, "\uacc4\uc7a5": {"personnel": "1", "period": "2", "unit_price": 144458.33333333334}, "\uc8fc\uc784": {"personnel": "", "period": "", "unit_price": 130916.66666666667}, "\uae30\uc0ac": {"personnel": "", "period": "", "unit_price": 121875.0}, "\uc5f0\uc7a5\uadfc\ubb34": {"personnel": "3", "period": "6", "unit_price": 4000.0}, "\uc57c\uac04\uadfc\ubb34": {"personnel": "", "period": "", "unit_price": 5000.0}, "\ud734\uc77c\uadfc\ubb34": {"personnel": "3", "period": "16.6667", "unit_price": 7500.0}}</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>[{"qty": "", "price": "2,200"}, {"qty": "", "price": "2,950"}, {"qty": "", "price": "2,700"}, {"qty": "", "price": "3,000"}, {"qty": "", "price": "2,600"}, {"qty": "", "price": "1,700"}, {"qty": "", "price": "100,000"}, {"qty": "", "price": "23,000"}, {"qty": "", "price": "23,000"}, {"qty": "", "price": "3,500"}, {"qty": "", "price": "10300000"}]</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>{"site_expense": [{"cat": "\ucc28\ub7c9\uc720\uc9c0\ube44", "cont": "\uc8fc\uc720, \uc218\ub9ac, \ud1b5\ud589, \uc8fc\ucc28 \ub4f1", "ppl": "4", "qty": "7", "unit": "\uc77c", "price": "6667", "amount": "46,669"}, {"cat": "\uc18c\ubaa8\ud488\ube44", "cont": "\uc7a5\uac11,\uc77c\ud68c\uc6a9 \uc791\uc5c5\ubcf5\uc678", "ppl": "N/A", "qty": "6", "unit": "\uac1c\uc6d4", "price": "100,000", "amount": "600,000"}, {"cat": "\ubcf5\ub9ac\ud6c4\uc0dd\ube44", "cont": "\uc0dd\uc218, \uc74c\ub8cc \uc678 \uae30\ud0c0", "ppl": "N/A", "qty": "6", "unit": "\uac1c\uc6d4", "price": "50,000", "amount": "300,000"}, {"cat": "Se-175", "cont": "\ubc29\uc0ac\uc131\ub3d9\uc704\uc6d0\uc18c \uad6c\ub9e4", "ppl": "N/A", "qty": "", "unit": "\uc77c", "price": "35,714", "amount": "0"}], "rental": [{"cat": "", "spec": "", "qty": "", "period": "", "unit": "", "price": "0", "amount": "0"}, {"cat": "", "spec": "", "qty": "", "period": "", "unit": "", "price": "0", "amount": "0"}, {"cat": "", "spec": "", "qty": "", "period": "", "unit": "", "price": "0", "amount": "0"}], "outsource": [{"cat": "\ucf00\uc774\uc5d4\ub514\uc774", "work": "\ubc29\uc0ac\uc120\ud22c\uacfc\uac80\uc0ac", "count": "0", "price": "0", "amount": "0"}, {"cat": "", "work": "", "count": "0", "price": "0", "amount": "0"}, {"cat": "", "work": "", "count": "0", "price": "0", "amount": "0"}], "depreciation": [{"item": "PAUT \uc7a5\ube44", "spec": "", "life": "5", "qty": "1", "days": "6", "rate": "44,444", "amount": "266,667"}, {"item": "PAUT SCANNER (MANUAL)", "spec": "", "life": "5", "qty": "1", "days": "6", "rate": "5,556", "amount": "33,333"}, {"item": "PAUT SCANNER (COBRA)", "spec": "", "life": "5", "qty": "1", "days": "", "rate": "16,667", "amount": "0"}, {"item": "YOKE", "spec": "", "life": "5", "qty": "1", "days": "", "rate": "222", "amount": "0"}, {"item": "\ud604\uc0c1\uc6a9 \ud0d1\ucc28(5\ub144\uac04 \ubcf4\ud5d8\ube44 \ud3ec\ud568)", "spec": "\ud604\uc7a5\ubcc4 \ucc28\ub7c9\uae30\uc785\uc2dc \ud0d1\ucc28 \uad6c\ubd84 \uae30\uc785", "life": "5", "qty": "1", "days": "", "rate": "16,667", "amount": "0"}, {"item": "\uc2a4\ud0c0\ub809\uc2a4(5\ub144\uac04 \ubcf4\ud5d8\ube44 \ud3ec\ud568)", "spec": "\ud604\uc7a5\ubcc4 \ucc28\ub7c9\uae30\uc785\uc2dc \uc2a4\ud0c0\ub809\uc2a4 \uad6c\ubd84 \uae30\uc785", "life": "5", "qty": "1", "days": "7", "rate": "16,667", "amount": "116,667"}], "_depreciation_precise_rates": [44444.441666666666, 5555.558333333333, 16666.666666666668, 222.2, 16666.666666666668, 16666.66875]}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix NDT truncation issues and sync Budget Tab perfectly with NDT Tab
</commit_message>
<xml_diff>
--- a/home/src/site_apps/central/data/Material_Inventory.xlsx
+++ b/home/src/site_apps/central/data/Material_Inventory.xlsx
@@ -26587,11 +26587,11 @@
         <v>480</v>
       </c>
       <c r="D7" t="n">
-        <v>17.8744</v>
+        <v>2.0385</v>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" s="1" t="n">
-        <v>46277.52000121528</v>
+        <v>46278.01189376158</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -26625,10 +26625,10 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>17.8744</v>
+        <v>2.0385</v>
       </c>
       <c r="Q7" t="n">
-        <v>201863</v>
+        <v>257675</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -26637,7 +26637,7 @@
         <v>0</v>
       </c>
       <c r="T7" t="n">
-        <v>3608180</v>
+        <v>525270</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
@@ -26787,7 +26787,7 @@
       </c>
       <c r="CC7" t="inlineStr">
         <is>
-          <t>300A 이상 (1.0)</t>
+          <t>200A (1.0)</t>
         </is>
       </c>
       <c r="CD7" t="inlineStr"/>
@@ -26797,19 +26797,19 @@
         <v>1</v>
       </c>
       <c r="CH7" t="n">
-        <v>17.8744</v>
+        <v>2.0385</v>
       </c>
       <c r="CI7" t="n">
-        <v>671344</v>
+        <v>76564</v>
       </c>
       <c r="CJ7" t="n">
-        <v>1165410</v>
+        <v>178058</v>
       </c>
       <c r="CK7" t="n">
-        <v>1281951</v>
+        <v>195863</v>
       </c>
       <c r="CL7" t="n">
-        <v>489472</v>
+        <v>74784</v>
       </c>
       <c r="CM7" t="inlineStr"/>
       <c r="CN7" t="inlineStr"/>
@@ -26827,14 +26827,14 @@
         </is>
       </c>
       <c r="CX7" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="CY7" t="n">
         <v>0</v>
       </c>
       <c r="CZ7" t="inlineStr">
         <is>
-          <t>700A</t>
+          <t>200A</t>
         </is>
       </c>
       <c r="DA7" t="inlineStr">
@@ -26862,11 +26862,11 @@
         <v>480</v>
       </c>
       <c r="D8" t="n">
-        <v>2.0385</v>
+        <v>17.8744</v>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" s="1" t="n">
-        <v>46277.52028597222</v>
+        <v>46278.01250546296</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -26900,7 +26900,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>2.0385</v>
+        <v>17.8744</v>
       </c>
       <c r="Q8" t="n">
         <v>201863</v>
@@ -26912,7 +26912,7 @@
         <v>0</v>
       </c>
       <c r="T8" t="n">
-        <v>411497</v>
+        <v>3608180</v>
       </c>
       <c r="U8" t="inlineStr">
         <is>
@@ -27072,19 +27072,19 @@
         <v>1</v>
       </c>
       <c r="CH8" t="n">
-        <v>2.0385</v>
+        <v>17.8744</v>
       </c>
       <c r="CI8" t="n">
-        <v>76564</v>
+        <v>671344</v>
       </c>
       <c r="CJ8" t="n">
-        <v>132910</v>
+        <v>1165410</v>
       </c>
       <c r="CK8" t="n">
-        <v>146201</v>
+        <v>1281951</v>
       </c>
       <c r="CL8" t="n">
-        <v>55822</v>
+        <v>489472</v>
       </c>
       <c r="CM8" t="inlineStr"/>
       <c r="CN8" t="inlineStr"/>
@@ -27102,14 +27102,14 @@
         </is>
       </c>
       <c r="CX8" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="CY8" t="n">
         <v>0</v>
       </c>
       <c r="CZ8" t="inlineStr">
         <is>
-          <t>200A</t>
+          <t>700A</t>
         </is>
       </c>
       <c r="DA8" t="inlineStr">

</xml_diff>